<commit_message>
Keep the catalogue spreadsheet's two copies in step
The copy beside the experiment folders was made by hand and went stale: it still
called experiment 07 "a perfect marker" after that was corrected to "the answer
key, no second model". The generator now writes both copies, and a test compares
them cell by cell.

Verified while checking systems 05/06/07: all three grade the same 1,319
attempt-1 answers and retry nothing, so all three correctly report 737 of 1,319
(55.88%). Every README and the CSV regenerated byte-identical.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01GnzEhGKwJZc4gVqTavue3g
</commit_message>
<xml_diff>
--- a/docs/experiments/benchmark_all_systems.xlsx
+++ b/docs/experiments/benchmark_all_systems.xlsx
@@ -587,7 +587,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:W20"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="46" customWidth="1" min="1" max="1"/>
     <col width="46" customWidth="1" min="2" max="2"/>
@@ -1201,12 +1201,12 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>A perfect marker marks every answer (the upper limit)</t>
+          <t>The answer key used as the marker (the upper limit)</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Verdict-only pass with the exact-match oracle</t>
+          <t>Verdict-only pass with the exact-match oracle; no second model is loaded</t>
         </is>
       </c>
       <c r="D8" t="n">
@@ -2207,7 +2207,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:C27"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="36" customWidth="1" min="1" max="1"/>
     <col width="100" customWidth="1" min="2" max="2"/>

</xml_diff>